<commit_message>
Verify Tier 1 prospect rows against Sep 2026 sources; swap Navan for Astera co-founder, add watch names
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYRxMiSxDbAaFrzq89rDxG
</commit_message>
<xml_diff>
--- a/docs/sales/bay-area-first-owner-prospects.xlsx
+++ b/docs/sales/bay-area-first-owner-prospects.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$L$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$L$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -555,22 +555,22 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Penngrove, Sonoma County</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>$3-6bn</t>
+          <t>$1.1bn (Forbes, Jun 2026; was $6.6bn at Aug 2025 peak)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Figma IPO Jul 2025; lock-up long expired; ongoing sales via 10b5-1</t>
+          <t>Figma IPO Jul 2025; regular 10b5-1 sales through 2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>No yacht on public record</t>
+          <t>No yacht on public record (verified Sep 2026)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -580,17 +580,17 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Personal office / Figma exec team; Iconiq-type manager likely</t>
+          <t>Personal office not public</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>First owner archetype: young, design-literate, will care about the build process. Sail or motor open.</t>
+          <t>First owner archetype: young, design-literate, will care about the build process. Stock fall since IPO means a 30-40m brief, not 50m.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Residence; whether a family office has been formed</t>
+          <t>Whether a family office has been formed</t>
         </is>
       </c>
     </row>
@@ -622,17 +622,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>$3-4bn</t>
+          <t>$3.2bn (Forbes, Sep 2026)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Meta's $14bn Scale stake Jun 2025 gave direct liquidity</t>
+          <t>Meta's $14.3bn purchase of 49% of Scale, Jun 2025, gave direct cash</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>No yacht on public record</t>
+          <t>No yacht on public record (verified Sep 2026)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -647,12 +647,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Cash liquid, mid-20s, high public profile. Time-poor; management plus OR bundle.</t>
+          <t>Cash liquid, 29, high public profile. Time-poor; management plus OR bundle.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Current residence (LA vs SF reported); appetite</t>
+          <t>Appetite</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>$3-5bn</t>
+          <t>$5.3-6.1bn (Forbes, 2026)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>No yacht on public record</t>
+          <t>No yacht on public record (verified Sep 2026)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>$2-3bn</t>
+          <t>$0.9-1bn (Forbes, Jul 2026)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Robinhood stock; sold down since 2024</t>
+          <t>Robinhood stock; sold down since 2024; put ~$10m into Aetherflux</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -870,12 +870,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>$1-1.5bn</t>
+          <t>$1.0bn (Forbes, Jul 2026)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Reddit IPO Mar 2024; ongoing stock sales</t>
+          <t>Reddit IPO Mar 2024; became a billionaire Nov 2025; regular sales</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -932,12 +932,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>$800m-1.5bn</t>
+          <t>~$700m (stake at CHYM $35, Sep 2026)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Chime IPO Jun 2025</t>
+          <t>Chime IPO Jun 2025; stock at $35 vs $26 float</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>$500m-1bn</t>
+          <t>~$650m (stake at CHYM $35, Sep 2026)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1036,32 +1036,32 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Ariel Cohen</t>
+          <t>Sanjay Gajendra</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Co-founder and CEO</t>
+          <t>Co-founder, President and COO</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Navan (travel and expense)</t>
+          <t>Astera Labs (AI connectivity)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Palo Alto</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>$300-700m</t>
+          <t>$1.7-2.5bn (Forbes, 2025-26)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Navan IPO Oct 2025</t>
+          <t>Astera Labs IPO Mar 2024; AI-cycle re-rating</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Israeli-born; travel-industry founder, likely Med charter familiarity.</t>
+          <t>Second Astera billionaire alongside Mohan; approach the pair through the same adviser.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Net worth after IPO performance; residence</t>
+          <t>Residence</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>$400-800m</t>
+          <t>~$305m (Jul 2026)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>$500m-1bn</t>
+          <t>Unclear: direct stake small, holdings via trusts; $47m single sale Sep 2025</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>$1-2bn</t>
+          <t>$2.0bn (Jul 2026)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>$500m-1.5bn</t>
+          <t>$3.2bn (Bloomberg, May 2026)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Cerebras IPO (2025-26); secondaries 2025</t>
+          <t>Cerebras IPO 14 May 2026 raised $5.5bn; lock-up expires ~Nov 2026</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1329,12 +1329,12 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Serial founder (SeaMicro exit to AMD). Liquidity newly real.</t>
+          <t>Serial founder (SeaMicro exit to AMD). The freshest large liquidity event on the list; approach adviser now, principal after lock-up.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>IPO completion and lock-up; net worth</t>
+          <t>Lock-up date; family office formation</t>
         </is>
       </c>
     </row>
@@ -1366,12 +1366,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>$2-4bn</t>
+          <t>$2bn+ (2026)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Databricks tenders 2024-26 at $60-100bn+; IPO expected</t>
+          <t>Databricks $190bn round Aug 2026 with employee tender; Ghodsi says no IPO in 2026</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Co-founder (Databricks, Anyscale); Professor</t>
+          <t>Co-founder and Executive Chairman (Databricks); Professor</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>$1-3bn</t>
+          <t>$5bn (Forbes, 2026; doubled in a year)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Databricks tenders</t>
+          <t>Databricks tenders 2025-26</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>$2-4bn</t>
+          <t>$2.3-3.4bn (2026)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>$1-2bn (paper)</t>
+          <t>$2.5bn (paper, Oct 2025)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Perplexity secondaries 2025-26</t>
+          <t>Perplexity valued $22.6bn Jan 2026; no personal secondary found</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Co-founder Character.AI; Google DeepMind</t>
+          <t>Co-founder Character.AI; VP Google DeepMind</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>$1-1.5bn</t>
+          <t>$0.6-1bn (2026)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Co-founder Instagram; Chief Product Officer, Anthropic</t>
+          <t>Co-founder Instagram; co-lead Anthropic Labs</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1676,12 +1676,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>$1-2bn</t>
+          <t>~$1bn (Aug 2026)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Instagram sale 2012; Anthropic equity re-rated 2025-26</t>
+          <t>Instagram sale 2012; Anthropic grant re-rated 2025-26</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>$2-3bn</t>
+          <t>$2.3bn (Forbes, Aug 2026)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>$9-12bn</t>
+          <t>$17.5bn (Aug 2026)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>$4-6bn</t>
+          <t>$5-6bn (Forbes, 2026)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2058,12 +2058,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Charters reported; no owned yacht on public record</t>
+          <t>No owned yacht on public record (Sep 2026 check: Hawaii megayacht stories were Orenstein and Maezawa, not Benioff)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Hawaii-based leisure; ocean affinity</t>
+          <t>Hawaii land; keeps an amphibious vehicle there; ocean affinity</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Santa Cruz coastal lifestyle</t>
+          <t>Santa Cruz coastal lifestyle; publicly said a giant yacht is 'not good for the planet'</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Post-CEO life, philanthropy-heavy; possible sail purchase. Medium priority.</t>
+          <t>Low priority: on record against big yachts. Only a sail or hybrid brief.</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>$1.5-2.5bn</t>
+          <t>$1.5bn (2026)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2792,12 +2792,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>$500m-1bn+</t>
+          <t>~$1bn (Forbes): $715m OpenAI stock vesting over years, ~$100m property, LoveFrom</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Apple; OpenAI acquired io for $6.5bn May 2025</t>
+          <t>Apple; OpenAI acquired io for $6.5bn May 2025; first device due late 2026</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>No superyacht on public record</t>
+          <t>No superyacht on public record (the 43m Benetti Diane is unrelated)</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -4624,8 +4624,194 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Greg Brockman</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder and President</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>~$30bn paper (own testimony, May 2026); $471m Stripe stake</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI IPO mooted late 2026; tenders ongoing</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>No yacht on public record</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>None known</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Personal office not public</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Largest paper fortune on the list; becomes a Tier 1 name the day OpenAI lists.</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>IPO timing; cash taken</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Mike Cagney</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder and Executive Chairman</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Figure Technology (blockchain lending); SoFi founder</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco (company HQ Reno)</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>$1.9bn (Bloomberg, Sep 2025)</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Figure IPO Sep 2025</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>No yacht on public record</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>None known</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Personal office not public</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Second public company; liquid. Residence needs confirming before treating as Bay Area.</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Residence</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Andy Rachleff</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder and Executive Chairman Wealthfront; Benchmark co-founder</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Wealthfront / VC</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Palo Alto</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>~$320m Wealthfront stake plus Benchmark wealth</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Wealthfront IPO Dec 2025</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>No yacht on public record</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>None known</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Personal office not public</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Older, established, teaches at Stanford GSB; brokerage 30m brief if any.</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Appetite</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L67"/>
+  <autoFilter ref="A1:L70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4636,7 +4822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4946,10 +5132,34 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
+          <t>Ariel Cohen (Navan)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Navan stock halved post-IPO; remaining stake in the tens of millions, below yacht scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>George Kurtz (CrowdStrike)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Took delivery of 80m Amels Pangea late 2025; Austin-based</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
           <t>Evan Spiegel</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
@@ -5104,7 +5314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -5120,33 +5330,47 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Basis: public profiles (Forbes, Bloomberg, IPO filings, press) to mid-2026. Live web verification was unavailable when the list was built, so net worth and residence entries are estimates and must be checked before any approach.</t>
+          <t>Basis: public profiles (Forbes, Bloomberg, IPO filings, press). Tier 1 net worth, residence and yacht status were checked against live sources on 10 Sep 2026; Tier 2 and 3 figures were spot-checked (Collison, Dorsey, Benioff, Ive, Greene, Hastings, Arora, Chesky, Camp, Larsen) and otherwise rest on 2025-26 public estimates.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>'No yacht on public record' means no ownership has been reported in the trade press or on the usual registries as far as known; it is not proof of non-ownership.</t>
+          <t>Verification findings 10 Sep 2026: Navan's Ariel Cohen removed (stake now tens of millions); Cerebras IPO completed 14 May 2026 (Feldman $3.2bn); Figma's Dylan Field down to $1.1bn; Ion Stoica up to $5bn; the two Hawaii megayacht stories of 2025-26 were Stephen Orenstein (Liva O) and Yusaku Maezawa (Nausicaa), not Benioff.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>No private contact details are held here. Route in via the public vehicles listed and the Routes in sheet.</t>
+          <t>Market note: the 100m Feadship Moonrise (ex Jan Koum) sold Jul 2026 through Burgess to an undisclosed buyer represented by Edmiston. If the buyer is a Bay Area name on this list, remove them.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Tier 1: recent liquidity, no known yacht, plausible purchase within 24 months. Tier 2: established liquid wealth, slower. Tier 3: investor wealth and watch list.</t>
+          <t>'No yacht on public record' means no ownership has been reported in the trade press or on the usual registries as far as known; it is not proof of non-ownership.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>No private contact details are held here. Route in via the public vehicles listed and the Routes in sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Tier 1: recent liquidity, no known yacht, plausible purchase within 24 months. Tier 2: established liquid wealth, slower. Tier 3: investor wealth and watch list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Excluded sheet lists Bay Area tech figures removed because they already own, have left the region, or are implausible buyers.</t>
         </is>

</xml_diff>

<commit_message>
Add Contacts sheet: published office and assistant routes for all 69 Bay Area prospects
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYRxMiSxDbAaFrzq89rDxG
</commit_message>
<xml_diff>
--- a/docs/sales/bay-area-first-owner-prospects.xlsx
+++ b/docs/sales/bay-area-first-owner-prospects.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes in" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes in" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$L$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contacts'!$A$1:$M$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -793,7 +795,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Co-founder (Robinhood); founder Aetherflux</t>
+          <t>Co-founder (Robinhood); founder and CEO Cowboy Space (formerly Aetherflux, $275m Series B May 2026)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1599,7 +1601,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Co-founder Character.AI; VP Google DeepMind</t>
+          <t>Co-founder Character.AI; reported moved to OpenAI Jun 2026</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2715,7 +2717,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Executive Chairman (from 1 Sep 2026; John Ternus CEO)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -3831,7 +3833,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Partner emeritus</t>
+          <t>Chairman (from Mar 2026)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -4817,6 +4819,4726 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M70"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vehicle to write to</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Vehicle URL</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Published email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Email source</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Named staff (public)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Staff source</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Email pattern (unverified)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Pattern source</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Office address (published)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Best route in</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dylan Field</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Figma, Inc. (no family office or foundation published)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.figma.com</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>press@figma.com; legal@figma.com</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>help.figma.com official-addresses article; figma.com/legal/privacy</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>functional inboxes only; no named example</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>help.figma.com</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Figma, Inc., 760 Market St, Floor 10, San Francisco, CA 94102; UK: Figma UK Ltd, 9 Devonshire Square, London EC2M 4YF</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Hard-copy letter to Dylan Field c/o Figma, 760 Market St Floor 10, marked personal and confidential</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Alexandr Wang</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Meta Platforms (Chief AI Officer); Scale AI (board). No family office published</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.meta.com/about/leadership/alexandr-wang/ ; https://scale.com</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>press@meta.com; Scale: privacy@scale.com only</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>about.fb.com/news press resources; scale.com/legal/privacy</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Meta Platforms, 1 Meta Way, Menlo Park, CA 94025; Scale AI, 650 Townsend Street, San Francisco, CA 94103</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Letter c/o Meta, 1 Meta Way, Menlo Park (Office of the Chief AI Officer); warm intro via Accel or Index more effective</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tony Xu</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>10x Better Foundation (private foundation with Patti Bao; no website). Otherwise DoorDash</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.givingpledge.org/pledger/patti-bao-and-tony-xu/ ; https://about.doordash.com</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>press@doordash.com; ir@doordash.com</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ir.doordash.com/resources/contact-us; DoorDash newsroom</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Patti Bao, Co-Chair and Treasurer, 10x Better Foundation</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Form 990 via Cause IQ (EIN 87-3883624)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>DoorDash, 303 2nd Street, Suite 800, San Francisco, CA 94107; foundation mailbox 2443 Fillmore St #346, San Francisco, CA 94115 (Form 990, unstaffed)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Letter jointly to Tony Xu and Patti Bao, 10x Better Foundation, at the Form 990 address; fallback c/o DoorDash HQ</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Vlad Tenev</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood Markets (Chairman and CEO); Harmonic (Executive Chairman, harmonic.fun). No family office published</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://robinhood.com/newsroom/ ; https://harmonic.fun</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>press@robinhood.com</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>press.robinhood.com</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood, 85 Willow Road, Menlo Park, CA 94025</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Vlad Tenev, Office of the CEO, Robinhood, 85 Willow Road, Menlo Park, marked personal and confidential</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Baiju Bhatt</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Cowboy Space Corporation (formerly Aetherflux; rebranded May 2026 with $275m Series B), founder and CEO</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cowboyspace.com</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>legal@cowboyspace.com (only address surfaced)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia article on Cowboy Space Corporation citing company legal pages; site has media kit only</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>functional@cowboyspace.com; no named example</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>legal@cowboyspace.com</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1710 Industrial Road, San Carlos, CA 94070 (lease reported by The Registry SF); site says San Carlos and Seattle</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Baiju Bhatt, Founder and CEO, Cowboy Space Corporation, 1710 Industrial Road, San Carlos</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Steve Huffman</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Reddit, Inc. No family office published</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://redditinc.com</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>press@reddit.com; licensing@reddit.com</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Reddit Help 'Press and Media' article</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Kevin Dious, Chief of Staff to CEO (LinkedIn headline per search index; unconfirmed)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/kdious</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Reddit, Inc., 303 2nd Street, South Tower, 5th Floor, San Francisco, CA 94104 (SEC EDGAR)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Steve Huffman c/o Kevin Dious, Chief of Staff to the CEO, Reddit, 303 2nd Street South Tower 5th Floor</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Chris Britt</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Chime Financial (CEO); founder of Chime Scholars Foundation. No family office published</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chime.com/press/ ; https://investors.chime.com</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>press@chime.com</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>chime.com/press Contact Us block (Cloudflare-obfuscated, decoded)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>none currently published (a Chief of Staff to CEO role existed in 2016)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>investors.chime.com management page</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>functional inbox only</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>chime.com/press</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Chime Financial, 101 California Street, Suite 500, San Francisco, CA 94111</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Chris Britt, Office of the CEO, Chime, 101 California Street Suite 500; or via Chime Scholars Foundation which he chairs</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ryan King</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Chime Financial (co-founder); angel investor; no fund or family office site verified</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chime.com</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>press@chime.com</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>chime.com/press</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Chime Financial, 101 California Street, Suite 500, San Francisco, CA 94111</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Ryan King, Co-founder, c/o Chime; joint approach with Britt through the same office</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Sanjay Gajendra</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Astera Labs (co-founder, President and COO). No family office published</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.asteralabs.com/company/contact-us/ ; https://ir.asteralabs.com</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>general contact email on asteralabs.com is obfuscated and could not be decoded; no IR email verified</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>asteralabs.com/company/contact-us</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Astera Labs, 2345 North First Street, San Jose, CA 95131 (HQ moved from Santa Clara)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Sanjay Gajendra, President and COO, Astera Labs, 2345 North First Street, San Jose; single letter to both founders</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Sanjay Beri</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Netskope Inc (founder and CEO). No family office published</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.netskope.com ; https://investors.netskope.com</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>none verified (contact pages 404, IR site timed out)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Netskope Inc, 2445 Augustine Drive, 3rd Floor, Santa Clara, CA 95054 (SEC EDGAR)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Sanjay Beri, Founder and CEO, Netskope, 2445 Augustine Drive 3rd Floor, Santa Clara</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Bipul Sinha</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Rubrik (Chairman and CEO); Venture Partner at Lightspeed with a published profile</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rubrik.com ; https://lsvp.com/team-member/bipul-sinha/</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>bipul@lsvp.com (on his official Lightspeed page); ir@rubrik.com</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>lsvp.com/team-member/bipul-sinha; ir.rubrik.com/resources/contact-ir</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Melissa Franchi, VP Investor Relations, Rubrik (corporate)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>ir.rubrik.com/resources/contact-ir</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>first@lsvp.com (demonstrated); Rubrik not demonstrable</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>lsvp.com/team-member/bipul-sinha</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Rubrik, 3495 Deer Creek Road, Palo Alto, CA 94304 (SEC filings)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Email bipul@lsvp.com, the address he publishes on his Lightspeed page; back up with letter to Rubrik HQ</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Jitendra Mohan</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Astera Labs (co-founder and CEO). No family office published</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.asteralabs.com/company/contact-us/ ; https://ir.asteralabs.com</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>none verified (obfuscated general address; IR site timed out)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>asteralabs.com/company/contact-us</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Astera Labs, 2345 North First Street, San Jose, CA 95131</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Jitendra Mohan, CEO, Astera Labs, 2345 North First Street, San Jose, jointly with Gajendra</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Andrew Feldman</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Cerebras Systems (co-founder and CEO; NASDAQ CBRS). No family office published</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cerebras.ai/contact ; https://investors.cerebras.ai</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>info@cerebras.ai; PR@zmcommunications.com (external media agency)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>cerebras.ai/contact-us; Cerebras press releases</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>functional inbox only</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>cerebras.ai/contact-us</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Cerebras Systems, 1237 E. Arques Ave, Sunnyvale, CA 94085</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Andrew Feldman, CEO, Cerebras, 1237 E. Arques Ave, Sunnyvale; Foundation Capital introduction is a credible warm route</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Ali Ghodsi</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Databricks (co-founder and CEO). No family office published</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.databricks.com/company/newsroom ; https://www.databricks.com/company/contact</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>press@databricks.com; partner-marketing@databricks.com</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>databricks.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>functional inboxes only</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>databricks.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Databricks, 160 Spear Street, 15th Floor, San Francisco, CA 94105; tel 1-866-330-0121</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Ali Ghodsi, Office of the CEO, Databricks, 160 Spear Street 15th Floor, marked personal and confidential</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Ion Stoica</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>UC Berkeley EECS / Sky Computing Lab (academic office); Databricks press office as alternative</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>https://www2.eecs.berkeley.edu/Faculty/Homepages/stoica.html ; https://sky.cs.berkeley.edu/contact/</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>istoica@cs.berkeley.edu (faculty); sky@cs.berkeley.edu (lab); press@databricks.com</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>vcresearch.berkeley.edu/faculty/ion-stoica; sky.cs.berkeley.edu/contact; databricks.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>EECS and Sky Lab pages list no admin staff</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Berkeley: first-initial+surname@cs.berkeley.edu (demonstrated). Databricks: none demonstrated</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>vcresearch.berkeley.edu/faculty/ion-stoica</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>481-2 Soda Hall; Sky Computing, UC Berkeley, 465 Soda Hall, MC-1776, Berkeley, CA 94720-1776. Databricks: 160 Spear Street, 15th Floor, San Francisco, CA 94105</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Academic-office letter to istoica@cs.berkeley.edu / 481-2 Soda Hall; Databricks press office fallback only</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Parker Conrad</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Rippling (company HQ)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rippling.com/press ; https://www.rippling.com/company/contact</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>press@rippling.com (media only)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>rippling.com/press</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Lia Duarte, Executive Assistant to CEO (org-chart sites only, not an official Rippling page)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>theorg.com; cbinsights.com</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>430 California Street, 11th Floor, San Francisco, CA 94105 (rippling.com/legal/privacy structured data)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Parker Conrad c/o Rippling, 430 California Street, 11th Floor, marked Office of the CEO</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Aravind Srinivas</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity AI</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perplexity.ai/help-center/en/articles/10354891-how-can-i-contact-the-perplexity-team</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>support@perplexity.ai; api@perplexity.ai. No press address confirmed (site 403)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity Help Center article per search summary</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>No usable direct channel; introduction via UC Berkeley network or investors</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Noam Shazeer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>none published. Reported (CNBC, 18 Jun 2026) to have left Google DeepMind for OpenAI; no family office found</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>none published (CNBC 2026-06-18 report)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Verify current employer (OpenAI per Jun 2026 reports); otherwise introduction via Character.AI or Google alumni</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Mike Krieger</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (co-lead, Labs)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/news</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>press@anthropic.com; support@anthropic.com</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>anthropic.com/news; anthropic.com/legal/consumer-terms</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>none published (co-leads Labs with Ben Mann, reporting to Daniela Amodei)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>The Information briefing</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic PBC, 548 Market Street, PMB 90375, San Francisco, CA 94104 (consumer terms mailbox)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Letter c/o Anthropic PBC, 548 Market Street PMB 90375, marked for Mike Krieger, Anthropic Labs</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Kevin Systrom</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Kevin and Nicole Systrom Foundation (private foundation, Palo Alto; no website)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>none published (https://projects.propublica.org/nonprofits/organizations/863372429)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Kevin Systrom, Co-president/Treasurer; Nicole Systrom, Co-president/Secretary (Form 990). No professional staff</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>ProPublica Nonprofit Explorer, EIN 86-3372429</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>none published (Palo Alto, CA only)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Introduction only, e.g. via Nicole Systrom's climate-philanthropy circles (Sutro Energy Group, Galvanize Climate) or Instagram-era co-investors</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Patrick Collison</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Stripe (CEO); Arc Institute (co-founder) as second door</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>https://stripe.com/newsroom ; https://arcinstitute.org/about</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>media@stripe.com; info@arcinstitute.org; donations@arcinstitute.org</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>stripe.com/newsroom; arcinstitute.org/about</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>none published. Arc Institute: Silvana Konermann, Co-Founder and Executive Director</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>arcinstitute.org/about</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>first@stripe.com (pattern, unverified; his X bio reportedly lists patrick@stripe.com)</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>x.com/patrickc per search results</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Stripe: 354 Oyster Point Boulevard, South San Francisco, CA 94080 (secondary sources). Arc Institute: Palo Alto</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Letter c/o Stripe, 354 Oyster Point Boulevard, South San Francisco, marked Office of the CEO</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Brian Chesky</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Airbnb (company HQ)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>https://news.airbnb.com/contact/</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>contact.press@airbnb.com (press)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>news.airbnb.com/contact</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>news.airbnb.com leadership pages</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>news.airbnb.com/contact</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>888 Brannan Street, San Francisco, CA 94103 (widely published)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Brian Chesky, Office of the CEO, Airbnb, 888 Brannan Street</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Nathan Blecharczyk</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Airbnb (Co-founder and Chief Strategy Officer); no family office found</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>https://news.airbnb.com/about-us/leadership/nathan-blecharczyk/</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>contact.press@airbnb.com (press only)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>news.airbnb.com/contact</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>888 Brannan Street, San Francisco, CA 94103</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Nathan Blecharczyk, Co-founder and CSO, Airbnb, 888 Brannan Street</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Jack Dorsey</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Block, Inc. (Block Head, Chairman); Start Small LLC has no official site; Iconiq reported wealth manager</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>https://investors.block.xyz/resources/contact/default.aspx</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>press@block.xyz; ir@block.xyz</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>investors.block.xyz/resources/contact</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>none published (Amrita Ahuja, Foundational Lead; Chrysty Esperanza, Counsel Lead; Owen Jennings, Business Lead)</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>investors.block.xyz/governance/leadership</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>none published (distributed company)</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ir@block.xyz or press@block.xyz asking to forward to the Block Head's office; or via Iconiq Capital</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Marc Benioff</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Time Ventures (family office; no reachable site). Salesforce (Chair and CEO) is the practical door</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com/company/leadership/</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>none published for Time Ventures</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>none published as chief of staff. Parker Harris listed as Co-Founder, Advisor to the CEO</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>salesforce.com/company/leadership</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce Tower, 415 Mission Street, 3rd Floor, San Francisco, CA 94105</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Marc Benioff, Office of the Chair and CEO, Salesforce Tower, 415 Mission Street</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Reed Hastings</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Powder Mountain (CEO and majority owner, Utah); Hastings Fund is a DAF at Silicon Valley Community Foundation</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.powdermountain.com/contact ; https://www.svcf.org/contact-us</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>support@powder.org; help@svcf.org; media@svcf.org</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>powdermountain.com/contact; svcf.org/contact-us</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Brandi Hammon, President, Powder Mountain (Nov 2025)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Press coverage (Fortune, Robb Report)</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Powder Mountain: 6965 E Powder Mountain Rd, Eden, UT 84310. SVCF: 444 Castro Street, Suite 140, Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Reed Hastings, CEO, Powder Mountain, via the President's office</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Jerry Yang</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>AME Cloud Ventures (Founding Partner)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amecloudventures.com/</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>pr@amecloudventures.com; contact@amecloudventures.com</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>amecloudventures.com homepage (obfuscated mailto links decoded from page source)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Cathy Luu, Operations Manager; Jeff Chung, Managing Director; Wretch Chien, Principal; Nick Adams, Venture Partner</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>amecloudventures.com team section</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Midtown Palo Alto (official site); 455B Portage Avenue, Palo Alto, CA 94306 per business directories</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Email contact@amecloudventures.com for Cathy Luu, Operations Manager, for Jerry Yang; pair with an introduction as the site prefers network approaches</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>David Filo</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Skyline Foundation (formerly Yellow Chair Foundation; David and Angela Filo)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>https://skylinefoundation.org/about/</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>info@skylinefoundation.org</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>skylinefoundation.org Contact Us mailto</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Angie Chen, Executive Director; Prizma Vazquez, Executive Assistant and Office Manager; Rose Brookhouse, Grants Manager; Raquel Donoso, Director of Programs</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>skylinefoundation.org/about</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrated</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1660 Bush Street, Suite 300, San Francisco, CA 94109 (foundation directories)</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Email info@skylinefoundation.org for Prizma Vazquez or Angie Chen asking for the letter to reach David Filo; frame as personal-office approach, not a grant</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Jayshree Ullal</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Arista Networks (Office of the CEO); no personal office published</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.arista.com</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>info@arista.com; ir@arista.com</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>arista.com/en/company/contact-us; investors.arista.com</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>none published (Investor Advocacy: Rudolph Araujo, Rod Hall, +1 408 547 8080)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Arista Q2 2026 press release</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>5453 Great America Parkway, Santa Clara, CA 95054</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Jayshree Ullal, President and CEO, c/o Arista HQ, marked personal; copy via info@arista.com for the office of the CEO</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Jay Chaudhry</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Zscaler (Office of the CEO). Jay and Jyoti Chaudhry Foundation (EIN 82-4247564, Atlanta) has no website</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zscaler.com</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>none published (web forms only)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>zscaler.com/company/contact; media-center</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>zscaler.com/company/leadership</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>120 Holger Way, San Jose, CA 95134; tel +1 408 533 0288</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Jay Chaudhry, Founder, Chairman and CEO, c/o Zscaler HQ, marked personal; Contact Us form as follow-up</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Ken Xie</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Fortinet (Office of the CEO); private Xie family foundation has no website</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fortinet.com</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>pr@fortinet.com; analystrelations@fortinet.com</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>fortinet.com/corporate/about-us/contact-us</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>fortinet.com executive-management page</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>909 Kifer Road, Sunnyvale, CA 94086; tel +1 408 235 7700</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Ken Xie, Founder, Chairman and CEO, c/o Fortinet HQ, marked personal; pr@fortinet.com to ask for the office of the CEO</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Aneel Bhusri</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Workday (Executive Chair's office); no family foundation, gives via Workday Foundation</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.workday.com</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>IR@workday.com; media@workday.com</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>investor.workday.com investor-contacts; newsroom.workday.com</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Justin Furby, VP Investor Relations (nearest published named contact)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>investor.workday.com/resource/investor-contacts</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>6110 Stoneridge Mall Road, Pleasanton, CA 94588; tel +1 925 951 9000</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Aneel Bhusri, Co-founder and Executive Chair, c/o Workday HQ, marked personal; IR@workday.com fallback</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Nikesh Arora</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Palo Alto Networks (Office of the Chairman and CEO)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.paloaltonetworks.com</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>press@paloaltonetworks.com</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>paloaltonetworks.com/company/newsroom</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>paloaltonetworks.com/about-us/management</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>3000 Tannery Way, Santa Clara, CA 95054</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Nikesh Arora, Chairman and CEO, c/o Palo Alto Networks HQ, marked personal</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Hock Tan</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Broadcom (Office of the President and CEO); Tan-Yang philanthropy via university centres, no foundation site</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.broadcom.com</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>none published (contact and IR pages returned no content)</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>broadcom.com/company/contact; investors.broadcom.com</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>broadcom.com executives page</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>HQ Palo Alto; verify 3421 Hillview Avenue, Palo Alto, CA 94304 before mailing</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Hock Tan, President and CEO, c/o Broadcom HQ Palo Alto, marked personal; IR web form only electronic route</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Jensen Huang</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA (Office of the CEO). Jen-Hsun and Lori Huang Foundation (EIN 26-1551239, c/o Frank Rimerman LLP, Palo Alto) has no website</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nvidia.com</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>press@nvidia.com; enterprise-pr@nvidia.com</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>nvidianews.nvidia.com/contacts</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>nvidianews.nvidia.com/bios and /contacts</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>2788 San Tomas Expressway, Santa Clara, CA 95051</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Jensen Huang, Founder, President and CEO, c/o NVIDIA HQ, marked personal; Frank Rimerman (foundation accountants) is a plausible adviser route</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Tim Cook</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Apple (Executive Chairman from 1 Sep 2026; John Ternus CEO). No personal office published</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apple.com</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>jrosenstock@apple.com (Josh Rosenstock, Apple press contact on the CEO-transition release)</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>apple.com/newsroom Apr 2026 CEO transition release, press contacts footer</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Josh Rosenstock, Apple communications (press contact). Cook's EA reported to remain in post but not named officially</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Apple Newsroom release; press coverage Aug 2026</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>first initial + surname @apple.com (pattern, unverified)</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>jrosenstock@apple.com on Apple Newsroom</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Apple, One Apple Park Way, Cupertino, CA 95014; tel +1 408 996 1010</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Tim Cook, Executive Chairman, c/o Apple Park, Cupertino, marked personal</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Sir Jony Ive</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>LoveFrom (with Marc Newson); io now within OpenAI</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lovefrom.com</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>none published (single text page, no contact details)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>lovefrom.com and lovefrom.com/jony</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Studio in Jackson Square, San Francisco; LoveFrom entities own 535 Pacific Avenue (SF Examiner, SFGate); registered mailing PO Box 471000, San Francisco, CA 94147 (California SoS filing for 535 Pacific, LLC)</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Sir Jony Ive c/o LoveFrom, 535 Pacific Avenue or PO Box 471000, San Francisco, CA 94147; physical letter is the only public channel</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Brian Armstrong</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Coinbase (remote-first, no HQ); brianarmstrong.org points to Coinbase, NewLimit, ResearchHub with no contact</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.coinbase.com ; https://www.brianarmstrong.org</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>investor@coinbase.com</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>investor.coinbase.com</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>none published (remote-first)</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>investor@coinbase.com or Coinbase press form addressed to the office of the CEO; no physical route published</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Fred Ehrsam</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Paradigm (co-founder; General Partner / Senior Advisor since Oct 2023)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.paradigm.xyz</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>info@paradigm.xyz; sf@paradigm.xyz; press@paradigm.xyz</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>paradigm.xyz/contact</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Katie Biber, COO; Alana Palmedo, Managing Partner</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>paradigm.xyz/team</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>none published (San Francisco, New York, Washington DC offices without street addresses)</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Email sf@paradigm.xyz addressed to Fred Ehrsam's office, copying Katie Biber, COO, by name</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Chris Larsen</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Rippleworks (co-founder, nonprofit with Doug Galen); Ripple Labs (Executive Chairman) as corporate route</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rippleworks.org ; https://ripple.com</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>none published (web forms only)</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>rippleworks.org/contact; ripple.com/contact/press</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Meeghan Zahorsky Paul, Chief of Staff, Rippleworks; Doug Galen, Co-Founder and CEO, Rippleworks</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>rippleworks.org/our-team</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Rippleworks: 585 Broadway, Redwood City, CA 94063 (Cause IQ registry)</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Chris Larsen c/o Rippleworks, Redwood City, attention Meeghan Zahorsky Paul, Chief of Staff; contact form as follow-up</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Garrett Camp</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Expa (founder and CEO); Camp.org (The Camp Foundation)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.expa.com ; https://camp.org</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>hello@expa.com; info@camp.org</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>expa.com home and about; camp.org</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>expa.com/about; garrettcamp.com</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Expa notice address 8605 Santa Monica Blvd, Suite #79245, West Hollywood, CA 90069 (mailbox); no SF street address published</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Email hello@expa.com addressed to Garrett Camp's office; letter via the Expa notice address as backup</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Evan Williams</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Obvious Ventures (co-founder); Chairman of Mozi and Medium</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>https://obvious.com</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>none on official site (newsletter form only)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>obvious.com and obvious.com/about</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Nett, Chief of Staff; Anico Steffen, Senior Executive Assistant; McKenzie Quinn, Executive Assistant; Cristina Kilmartin, Office Manager; Sarah Beresford, Head of Investor Relations</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>obvious.com/team</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>190 Pacific Avenue, San Francisco, CA 94111</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Ev Williams c/o Obvious Ventures, 190 Pacific Avenue, attention Jessica Nett, Chief of Staff</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Ben Silbermann</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Pinterest, Inc. (Executive Chair). No family office published</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>https://newsroom.pinterest.com/ ; https://investor.pinterestinc.com/</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>press@pinterest.com (press and speaker requests only)</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>newsroom.pinterest.com/contact</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Pinterest newsroom, IR governance pages</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Pinterest HQ, 651 Brannan Street, San Francisco, CA 94107 (SEC filings)</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Pinterest HQ for the Office of the Executive Chair; warm intro via a founder he backs or Benchmark is more realistic</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Jeff Lawson</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Global Tetrahedron LLC (owner of The Onion; Lawson is Owner and Chairman). No family office site found</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>https://theonion.com/about-us/</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>press@theonion.com; legal@theonion.com; marketing@theonion.com</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>theonion.com/about-us</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Ben Collins, CEO, The Onion; Paula Brillson, Counsel</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>theonion.com/about-us masthead</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>none published (Global Tetrahedron is Chicago-based)</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Email press@theonion.com or legal@theonion.com asking for forwarding to the Office of the Chairman; or via Ben Collins as CEO</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Zhao</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Notion Labs, Inc. (CEO). No personal vehicle published</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.notion.com/</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>team@makenotion.com (Crunchbase listing, not confirmed on notion.com; press page 404)</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Crunchbase company profile</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>notion.com about page</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>makenotion.com is the corporate mail domain (pattern, unverified)</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>team@makenotion.com</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>none published; 'downtown San Francisco'</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Notion HQ for the Office of the CEO; warm intro via Sequoia or Index more realistic</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Max Levchin</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>SciFi VC (personal venture fund of Max and Nellie Levchin); also Affirm (CEO)</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>https://scifi.vc/</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>info@scifi.vc</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>scifi.vc homepage contact section</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Mikaela Encarnacion, Executive Assistant; Matt Therian, Partner, Finance and Operations; Brooks Hosfield, Partner (formerly Chief of Staff to Levchin)</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>scifi.vc team listing</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>none published on scifi.vc (San Francisco). Affirm HQ 650 California Street, San Francisco, CA 94108</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Email info@scifi.vc for the attention of Mikaela Encarnacion, Executive Assistant. Best-published personal-office channel in this batch</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Mark Pincus</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Reinvent Capital (Co-founder and Managing Member); Playful.AI founder</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>https://reinventcapital.com/</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>email@reinventcapital.com</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>reinventcapital.com contact field</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>none currently published; a Jan 2026 recruiter post says Pincus is hiring a Chief of Staff covering new companies, investments and foundation</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn post by recruiter Katie Kirsch, Jan 2026</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Email email@reinventcapital.com for the attention of Mark Pincus's office; re-check in a few months for the new chief of staff</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Diane Greene</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>No family office or foundation published for Greene and Mendel Rosenblum. Chair of the MIT Corporation</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>https://corporation.mit.edu/</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>corporationoffice@mit.edu (institutional, not her personal office)</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>corporation.mit.edu/contact</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>searches returned nothing</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>MIT Corporation office, Room 7-203, 77 Massachusetts Avenue, Cambridge, MA 02139; tel 617 253 5614. No Bay Area office published</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Letter via the MIT Corporation office addressed to the Chair, or warm intro through VMware or Google Cloud alumni; StFYC route worth testing given her sailing history</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Scott Cook</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Fox Hollow Ventures LLC (single family office for Scott Cook and Signe Ostby, Woodside; no website) and Valhalla Foundation (same office)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>https://valhalla.org/</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>info@valhalla.org (site states no unsolicited funding requests)</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>valhalla.org homepage mailto (decoded)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Sara Allan, President; Alex Terman, MD Finance and Operations; Lynne Durie, Executive Assistant; Prudence Chikono, Executive Assistant</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>valhalla.org/people</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>2995 Woodside Road, Suite 400, Woodside, CA 94062 (EPIP/Candid listings)</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Fox Hollow Ventures / Valhalla Foundation, 2995 Woodside Road Suite 400, for the Executive Assistant to Scott Cook, backed by email to info@valhalla.org</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Tom Siebel</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Thomas and Stacey Siebel Foundation and First Virtual Group (holding company, Chairman), Redwood City</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siebelfoundation.org/ (unreachable this session) ; https://www.siebelscholars.com/</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>ssf@siebel.org; tel +1 650 299 5200</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>siebelscholars.com/contact</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>siebelscholars.com/contact</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>siebel.org shared office domain (pattern, unverified)</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>ssf@siebel.org</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>1400 Seaport Blvd, Suite 301A, Redwood City, CA 94063 (Siebel Scholars); foundation registered at 1300 Seaport Blvd, Suite 400</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Thomas M. Siebel, Chairman, First Virtual Group / Siebel Foundation, 1400 Seaport Blvd Suite 301A, copy to ssf@siebel.org</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Vinod Khosla</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Khosla Ventures</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.khoslaventures.com/</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>kv@khoslaventures.com; media@khoslaventures.com</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>khoslaventures.com/contact</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Nicole Mihelson, Chief of Staff to Vinod Khosla (since 2023); Hari Arul, former Chief of Staff, now on KV team</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>theorg.com; khoslaventures.com/team/hari-arul</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>2128 Sand Hill Road, Menlo Park, CA 94025; tel 650 376 8500</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Letter or email to kv@khoslaventures.com marked for Nicole Mihelson, Chief of Staff to Vinod Khosla</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>John Doerr</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Kleiner Perkins (Chairman). Benificus Foundation (Ann Doerr, President) has no website</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kleinerperkins.com/people/advisors/john-doerr/</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>none published (no contact or press page)</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>kleinerperkins.com</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>2750 Sand Hill Road, Menlo Park, CA 94025; tel +1 650 233 2750 (PEI profile)</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Kleiner Perkins, 2750 Sand Hill Road, for the Office of John Doerr, Chairman</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Sir Michael Moritz</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Crankstart (family foundation of Moritz and Harriet Heyman; philanthropic, not investment)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>https://crankstart.org/</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>communications@crankstart.org; general inquiries via web form</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>crankstart.org/contact</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Missy Narula, CEO; Eli Bildner, VP Operations; Kristin McCann, Executive Assistant; Carol Kim, Director of Finance</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>crankstart.org/team</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Crankstart c/o Pacific Foundation Services, 1660 Bush St #300, San Francisco, CA 94109</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Crankstart c/o Pacific Foundation Services for Kristin McCann, Executive Assistant, or Missy Narula, CEO</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Doug Leone</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Sequoia Capital (named Chairman, Mar 2026). No personal vehicle published</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>https://sequoiacap.com/people/doug-leone</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>sequoiacap.com</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Sequoia Capital, 2800 Sand Hill Road, Suite 101, Menlo Park, CA 94025 (widely published)</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Sequoia Capital, 2800 Sand Hill Road, for the Office of Doug Leone, Chairman</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Marc Andreessen</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Andreessen Horowitz (a16z)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>https://a16z.com/</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>menlopark-info@a16z.com; sanfrancisco-info@a16z.com</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>a16z.com/offices</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>a16z.com/offices; jobs.a16z.com</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>2865 Sand Hill Road, Suite 101, Menlo Park, CA 94025; 180 Townsend Street, San Francisco, CA 94107</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Email menlopark-info@a16z.com and letter to 2865 Sand Hill Road Suite 101, for the Office of Marc Andreessen</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>David Sacks</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Craft Ventures (Co-founder; currently White House AI and Crypto adviser, reported stepped back from day-to-day)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.craftventures.com/</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>craftventures.com</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Brunt, Operating Partner, Chief of Staff to David Sacks; Brian Murray, Partner and COO; Mark Woolway, President; Caroline Brayson, Operating Partner, Communications</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>craftventures.com/team</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>855 Front Street, San Francisco, CA 94111 (craft.co profile)</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Craft Ventures, 855 Front Street, for Daniel Brunt, Chief of Staff to David Sacks</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Chamath Palihapitiya</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Social Capital</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.socialcapital.com/</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>inbox@socialcapital.com (pitch inbox, not on the official site)</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>superscout.co investor guide; official site publishes no email</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>socialcapital.com/about</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>317 University Ave, Suite 200, Palo Alto, CA 94301 (SEC S-1, 2020)</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Letter c/o Social Capital, 317 University Ave Suite 200, Palo Alto, copy to inbox@socialcapital.com</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Tim Draper</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Draper Associates</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.draper.vc/</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>andy@draper.vc (LP inquiries); no general inbox</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>draper.vc/contact</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Addie Bonifas, Chief of Staff; Tatiana Chau, Chief of Staff to Andy Tang; Rose Yip, CFO; Staci Robilio, Executive Assistant (org-chart listings)</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>draper.vc/team; theorg.com for Robilio</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>first@draper.vc (pattern, unverified)</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>andy@draper.vc on draper.vc/contact</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>55 E 3rd Ave, San Mateo, CA 94401; tel 650-963-6339</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Tim Draper c/o Addie Bonifas, Chief of Staff, Draper Associates, 55 E 3rd Ave, San Mateo</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Ron Conway</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>SV Angel</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>https://svangel.com/</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>svangel.com publishes no email or address</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Zachary Miller, COO; Paulina Briones, Executive Assistant; Diana Duane, Office Manager</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>svangel.com/about/team</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>none on site; third-party: 588 Sutter St, Suite 299, San Francisco, CA 94102 (unverified)</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Ron Conway c/o Zachary Miller, COO, SV Angel; or LinkedIn approach to the COO/EA</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Ram Shriram</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Sherpalo Ventures</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sherpalo.com/</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>none published (site asks for email submissions but shows no address in fetched pages)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>sherpalo.com</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>none published ('very limited staffing')</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>sherpalo.com</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>none published; Menlo Park, CA</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Locate the contact link on sherpalo.com; otherwise letter c/o Sherpalo Ventures, Menlo Park</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Joe Lacob</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Golden State Warriors / Chase Center</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nba.com/warriors/</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>publicrelations@warriors.com; guestexperiences@warriors.com</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>chasecenter.com A-to-Z Guide</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>nba.com/warriors/staff/joe-lacob</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Chase Center, 1 Warriors Way, San Francisco, CA 94158</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Joe Lacob, Co-Executive Chairman and CEO, c/o Golden State Warriors, Chase Center, flagged to publicrelations@warriors.com</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Sheryl Sandberg</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Sandberg Goldberg Bernthal Family Foundation (Lean In / Option B)</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>https://sgb.org/ ; https://leanin.org/</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>info@leanin.org; press@leanin.org; partners@leanin.org</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>leanin.org/about/contact/</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Katie DiClemente, Chief of Staff, Office of the Founder; Bridget Griswold, CEO; Brandon McCormick, VP Communications</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>sgb.org/team</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>PO Box 26221, San Francisco, CA 94126</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Sheryl Sandberg c/o Katie DiClemente, Chief of Staff, SGB Family Foundation, PO Box 26221, San Francisco, copy to info@leanin.org</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Reid Hoffman</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Greylock Partners (also reidhoffman.org, Manas AI)</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>https://greylock.com/</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>press@greylock.com</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>greylock.com/contact-us/ (tel 650-493-5525)</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Aria Finger, Chief of Staff to Reid Hoffman</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>ariafinger.com; Forbes 15 Nov 2022</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>first-initial+last@greylock.com (pattern, unverified)</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>vcsheet.com listing; not published by Greylock</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>2550 Sand Hill Road, Suite 200, Menlo Park, CA 94025; 140 New Montgomery St, Suite 2600, San Francisco, CA 94105</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Reid Hoffman c/o Aria Finger, Chief of Staff, Greylock Partners, 2550 Sand Hill Road Suite 200, Menlo Park</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Elad Gil</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Gil and Co (multi-stage investment firm)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>https://eladgil.com/</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>eladgil.com carries no email; X and Substack only</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>search results</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>none published; San Francisco</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>Warm introduction only, or short note via X/Substack</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Dario Amodei</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic PBC</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>press@anthropic.com; support@anthropic.com</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic press materials; anthropic.com/legal/consumer-terms</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Avital Balwit, Chief of Staff to Dario Amodei</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>avitalbalwit.com; Fortune 18 Jun 2026; TechCrunch 10 Jun 2026</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic PBC, 548 Market Street, PMB 90375, San Francisco, CA 94104-5401; tel (415) 326-6303</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Dario Amodei c/o Avital Balwit, Chief of Staff, Anthropic PBC, 548 Market Street PMB 90375, copy to press@anthropic.com</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Sam Altman</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI (Hydrazine Capital has no site or published contact)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>https://openai.com/</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>press@openai.com</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI announcements and Newsroom</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>none verified (openai.com policy pages 403); HQ San Francisco, Mission Bay</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Sam Altman, Office of the CEO, c/o OpenAI, San Francisco, flagged to press@openai.com</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Greg Brockman</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>https://openai.com/</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>press@openai.com</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI announcements and Newsroom</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>CNBC 10 Jul 2026; Axios 14 Aug 2026 name no chief of staff</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>none verified</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Greg Brockman, President, c/o OpenAI, San Francisco, flagged to press@openai.com</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Mike Cagney</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Figure Technology Solutions (NASDAQ: FIGR)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.figure.com/ ; https://investors.figure.com/</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>press@figure.com; investors@figure.com</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>figure.com/newsroom; GlobeNewswire release 3 Sep 2026</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>investors.figure.com board page</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>650 California Street, Suite 2700, San Francisco, CA 94108; tel (628) 210-6937 (SEC filing)</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Mike Cagney, Executive Chairman, c/o Figure, 650 California Street Suite 2700, copy to press@figure.com</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Andy Rachleff</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Wealthfront Corporation</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wealthfront.com/</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>none published (support line 844-995-8437 only)</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>wealthfront.com/contact-us; wealthfront.com/legal/disclosure</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>wealthfront.com/blog/author/andy/</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>none demonstrable</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>none published</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>none on site; third-party: 261 Hamilton Ave, Palo Alto, CA 94301 (unverified)</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Letter to Andy Rachleff, Executive Chairman, c/o Wealthfront, Palo Alto; or via Stanford GSB</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M70"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5170,7 +9892,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5308,7 +10030,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>